<commit_message>
Small changes for PR
</commit_message>
<xml_diff>
--- a/test/configs/data/develop/2n_1c_1g_1h.xlsx
+++ b/test/configs/data/develop/2n_1c_1g_1h.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" activeTab="2"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Carrier" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="135">
   <si>
     <t>name</t>
   </si>
@@ -428,6 +428,9 @@
   </si>
   <si>
     <t>IT0 1</t>
+  </si>
+  <si>
+    <t>line 0-1</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1210,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="4" width="8.88671875" style="5" bestFit="1" customWidth="1"/>
@@ -1239,6 +1242,32 @@
       </c>
       <c r="H1" s="9" t="s">
         <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="5">
+        <v>5</v>
+      </c>
+      <c r="G2" s="5">
+        <v>0.1</v>
+      </c>
+      <c r="H2" s="5">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>